<commit_message>
tests , multi-browser <parallel Tests> done
</commit_message>
<xml_diff>
--- a/groceryproject/src/test/resources/TestData.xlsx
+++ b/groceryproject/src/test/resources/TestData.xlsx
@@ -3,18 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{6811E6A4-6CEC-4080-B939-2659D2462A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{8F420D61-8BBC-4461-90D4-FE1FE8876EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{629CD4EF-AB6C-44C5-A0B3-A2D5706B26C8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{629CD4EF-AB6C-44C5-A0B3-A2D5706B26C8}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPage" sheetId="1" r:id="rId1"/>
     <sheet name="NewsPage" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="4" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId4"/>
+    <sheet name="AdminPage" sheetId="4" r:id="rId3"/>
+    <sheet name="FooterTextPage" sheetId="6" r:id="rId4"/>
+    <sheet name="ContactPage" sheetId="7" r:id="rId5"/>
+    <sheet name="Sheet3" sheetId="5" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:M8"/>
+  <oleSize ref="A1:Q9"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="19">
   <si>
     <t>Username</t>
   </si>
@@ -45,16 +48,60 @@
   </si>
   <si>
     <t>Snow1 alert</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Pwd</t>
+  </si>
+  <si>
+    <t>adtestadmin</t>
+  </si>
+  <si>
+    <t>Staff</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>test@yopmail.com</t>
+  </si>
+  <si>
+    <t>CT</t>
+  </si>
+  <si>
+    <t>DCT</t>
+  </si>
+  <si>
+    <t>testcontact@yopmail.com</t>
+  </si>
+  <si>
+    <t>testcontact Address</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -77,13 +124,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -485,6 +535,129 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69FC2C9A-538A-424F-946D-714A7C0E8BE5}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99738129-867F-48D4-9AD8-C79B170FC1DD}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="18.44140625" customWidth="1"/>
+    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>894444431</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{FAC3460F-8779-40B0-8603-BF3F741A3504}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6682C4C3-9061-4BAD-83BA-68F4AFDEC561}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.77734375" customWidth="1"/>
+    <col min="3" max="3" width="29.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>892367739</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{7D6A4518-1467-4BAC-A946-5CB923CB0567}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B04E6E56-E156-4483-B1B7-D6F6E582C08F}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
@@ -492,7 +665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF5C660F-9D00-4D57-A435-325262B51999}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>